<commit_message>
update schedule file to reflect latest changes
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C091B908-C604-4E9F-94B8-9396A2195CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64B175E-6D26-4C90-84F1-F0FA24B5A26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="120">
   <si>
     <t>Class number</t>
   </si>
@@ -223,9 +223,6 @@
     <t>1. Classical search</t>
   </si>
   <si>
-    <t>8. Final project</t>
-  </si>
-  <si>
     <t>ThinkingAI5-7</t>
   </si>
   <si>
@@ -284,9 +281,6 @@
   </si>
   <si>
     <t xml:space="preserve">6. Transformers and large language models </t>
-  </si>
-  <si>
-    <t>HW5&amp;6</t>
   </si>
   <si>
     <t>Q5&amp;6</t>
@@ -521,6 +515,15 @@
   </si>
   <si>
     <t>Computationalism</t>
+  </si>
+  <si>
+    <t>updated 9/12/2026</t>
+  </si>
+  <si>
+    <t>HW6</t>
+  </si>
+  <si>
+    <t>7. Final project</t>
   </si>
 </sst>
 </file>
@@ -911,27 +914,78 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -946,57 +1000,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1306,20 +1309,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.453125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7265625" style="38" customWidth="1"/>
-    <col min="9" max="9" width="37.81640625" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" style="38" customWidth="1"/>
+    <col min="9" max="9" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -1336,18 +1339,18 @@
         <v>0</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G1" s="42" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H1" s="43" t="s">
         <v>42</v>
       </c>
       <c r="I1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="46">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="47">
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
@@ -1356,7 +1359,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="49" t="s">
+      <c r="D2" s="65" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1364,12 +1367,12 @@
       </c>
       <c r="F2" s="10"/>
       <c r="G2" s="21" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H2" s="33"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="47"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="48"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
       </c>
@@ -1377,20 +1380,20 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="50"/>
+      <c r="D3" s="67"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="21" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H3" s="33" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="46">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="47">
         <f>A2+1</f>
         <v>2</v>
       </c>
@@ -1402,18 +1405,18 @@
         <f>C2+7</f>
         <v>46273</v>
       </c>
-      <c r="D4" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
+      <c r="D4" s="53" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
       <c r="G4" s="21"/>
       <c r="H4" s="33" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="47"/>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="48"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
         <v>Fri</v>
@@ -1422,24 +1425,24 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="68" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H5" s="33" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="46">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="47">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
       </c>
@@ -1451,7 +1454,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="45"/>
+      <c r="D6" s="68"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1459,14 +1462,14 @@
         <v>43</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H6" s="33" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="47"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="48"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1476,21 +1479,21 @@
         <v>46283</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H7" s="33" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="46">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="47">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
       </c>
@@ -1502,24 +1505,24 @@
         <f t="shared" si="2"/>
         <v>46287</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="68" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H8" s="33" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="47"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="48"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1528,7 +1531,7 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="45"/>
+      <c r="D9" s="68"/>
       <c r="E9" s="5" t="s">
         <v>11</v>
       </c>
@@ -1536,53 +1539,53 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="46">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="47">
         <f>A8+1</f>
         <v>5</v>
       </c>
-      <c r="B10" s="46" t="str">
+      <c r="B10" s="47" t="str">
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="52">
+      <c r="C10" s="69">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="49" t="s">
-        <v>61</v>
+      <c r="D10" s="65" t="s">
+        <v>60</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="48"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="57" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" s="58"/>
-      <c r="G11" s="58"/>
-      <c r="H11" s="59"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="47"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="52"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="50"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="51"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="48"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
         <v>Fri</v>
@@ -1591,22 +1594,22 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="71"/>
+      <c r="D12" s="66"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="46">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="47">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
       </c>
@@ -1618,20 +1621,20 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="50"/>
+      <c r="D13" s="67"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H13" s="33"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="47"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="48"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1650,12 +1653,12 @@
         <v>45</v>
       </c>
       <c r="G14" s="44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H14" s="33"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="46">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="47">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
       </c>
@@ -1675,12 +1678,12 @@
       </c>
       <c r="F15" s="10"/>
       <c r="G15" s="44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H15" s="34"/>
     </row>
-    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="47"/>
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="48"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1690,20 +1693,20 @@
         <v>46311</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1716,13 +1719,13 @@
       <c r="D17" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="54"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="56"/>
-    </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" s="46">
+      <c r="E17" s="71"/>
+      <c r="F17" s="72"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="73"/>
+    </row>
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="47">
         <v>8</v>
       </c>
       <c r="B18" s="16" t="str">
@@ -1733,7 +1736,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="68" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1741,66 +1744,66 @@
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="48"/>
-      <c r="B19" s="67" t="str">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="52"/>
+      <c r="B19" s="61" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="69">
+      <c r="C19" s="63">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="45"/>
+      <c r="D19" s="68"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="47"/>
-      <c r="B20" s="68"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="64" t="s">
-        <v>86</v>
-      </c>
-      <c r="F20" s="65"/>
-      <c r="G20" s="65"/>
-      <c r="H20" s="66"/>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="46">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="48"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="60"/>
+    </row>
+    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="47">
         <v>9</v>
       </c>
       <c r="B21" s="39" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C21" s="40">
         <v>46324</v>
       </c>
-      <c r="D21" s="45"/>
-      <c r="E21" s="51" t="s">
-        <v>88</v>
-      </c>
-      <c r="F21" s="51"/>
-      <c r="G21" s="51"/>
-      <c r="H21" s="51"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="48"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="52"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1809,20 +1812,20 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="45"/>
+      <c r="D22" s="68"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H22" s="33" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="47"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="48"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
         <v>Tue</v>
@@ -1832,21 +1835,21 @@
         <v>46329</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="25"/>
       <c r="G23" s="21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="46">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="47">
         <v>10</v>
       </c>
       <c r="B24" s="16" t="str">
@@ -1864,15 +1867,15 @@
         <v>22</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H24" s="33"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="47"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="48"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -1881,41 +1884,41 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="45" t="s">
-        <v>65</v>
+      <c r="D25" s="68" t="s">
+        <v>64</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H25" s="34"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="60">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="54">
         <f>A24+1</f>
         <v>11</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="45"/>
-      <c r="E26" s="63" t="s">
-        <v>90</v>
-      </c>
-      <c r="F26" s="63"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="63"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="61"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="57" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="55"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -1924,20 +1927,20 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="45"/>
+      <c r="D27" s="68"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="62"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="56"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -1947,21 +1950,21 @@
         <v>46343</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="21"/>
       <c r="G28" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H28" s="33" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="46">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="47">
         <f>A26+1</f>
         <v>12</v>
       </c>
@@ -1974,21 +1977,21 @@
         <v>46346</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>49</v>
+        <v>119</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G29" s="44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H29" s="34"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="47"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="48"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2004,16 +2007,16 @@
         <v>27</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
       <c r="G30" s="44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H30" s="33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2031,8 +2034,8 @@
       <c r="G31" s="21"/>
       <c r="H31" s="33"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="46">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="47">
         <f>A29+1</f>
         <v>13</v>
       </c>
@@ -2052,12 +2055,12 @@
       </c>
       <c r="F32" s="10"/>
       <c r="G32" s="44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H32" s="36"/>
     </row>
-    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="47"/>
+    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="48"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2067,24 +2070,24 @@
         <v>46360</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="G33" s="72" t="s">
-        <v>104</v>
+        <v>66</v>
+      </c>
+      <c r="G33" s="45" t="s">
+        <v>102</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I33"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="46">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="47">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
       </c>
@@ -2097,21 +2100,21 @@
         <v>46364</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F34" s="19"/>
       <c r="G34" s="41" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H34" s="33" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="47"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="48"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2121,20 +2124,20 @@
         <v>46367</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>31</v>
       </c>
       <c r="F35" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="G35" s="73" t="s">
-        <v>104</v>
+        <v>67</v>
+      </c>
+      <c r="G35" s="46" t="s">
+        <v>102</v>
       </c>
       <c r="H35" s="34"/>
     </row>
-    <row r="36" spans="1:9" ht="39" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="16" t="s">
         <v>35</v>
@@ -2143,24 +2146,43 @@
         <v>38</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="33"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F37" s="6"/>
       <c r="H37" s="37"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D38" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D39"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E17:H17"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2177,20 +2199,6 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E17:H17"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix formatting in HW6 assignment index
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64B175E-6D26-4C90-84F1-F0FA24B5A26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F141D352-EC8D-42F3-938C-123F2E056030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="124">
   <si>
     <t>Class number</t>
   </si>
@@ -223,12 +223,6 @@
     <t>1. Classical search</t>
   </si>
   <si>
-    <t>ThinkingAI5-7</t>
-  </si>
-  <si>
-    <t>ThinkingAI8-10</t>
-  </si>
-  <si>
     <t>ThinkingAI1-4 + Turing1950</t>
   </si>
   <si>
@@ -242,12 +236,6 @@
   </si>
   <si>
     <t>Q3</t>
-  </si>
-  <si>
-    <t>ThinkingAI11 + searle1980</t>
-  </si>
-  <si>
-    <t>ThinkingAI12-14</t>
   </si>
   <si>
     <t>[final project]</t>
@@ -525,6 +513,30 @@
   <si>
     <t>7. Final project</t>
   </si>
+  <si>
+    <t>D1: ThinkingAI5-7</t>
+  </si>
+  <si>
+    <t>D2: ThinkingAI8-10</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3: ThinkingAI11 + searle1980</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D4: ThinkingAI12-14</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
 </sst>
 </file>
 
@@ -533,7 +545,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -559,14 +571,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -845,7 +849,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -854,9 +858,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -908,7 +909,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
@@ -920,25 +921,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -974,31 +999,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1318,7 +1322,7 @@
     <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
     <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7109375" style="38" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" style="37" customWidth="1"/>
     <col min="9" max="9" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1332,19 +1336,19 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="G1" s="42" t="s">
-        <v>93</v>
-      </c>
-      <c r="H1" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="41" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="42" t="s">
         <v>42</v>
       </c>
       <c r="I1"/>
@@ -1359,7 +1363,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="65" t="s">
+      <c r="D2" s="50" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1367,9 +1371,9 @@
       </c>
       <c r="F2" s="10"/>
       <c r="G2" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="H2" s="33"/>
+        <v>87</v>
+      </c>
+      <c r="H2" s="32"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="48"/>
@@ -1380,16 +1384,16 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="67"/>
+      <c r="D3" s="51"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="H3" s="33" t="s">
-        <v>104</v>
+        <v>88</v>
+      </c>
+      <c r="H3" s="32" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1405,14 +1409,14 @@
         <f>C2+7</f>
         <v>46273</v>
       </c>
-      <c r="D4" s="53" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
+      <c r="D4" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
       <c r="G4" s="21"/>
-      <c r="H4" s="33" t="s">
-        <v>89</v>
+      <c r="H4" s="32" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1425,20 +1429,20 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="68" t="s">
+      <c r="D5" s="46" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="H5" s="33" t="s">
-        <v>105</v>
+        <v>91</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1454,7 +1458,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="68"/>
+      <c r="D6" s="46"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1462,10 +1466,10 @@
         <v>43</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="H6" s="33" t="s">
         <v>90</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1478,18 +1482,18 @@
         <f t="shared" si="2"/>
         <v>46283</v>
       </c>
-      <c r="D7" s="28" t="s">
-        <v>51</v>
+      <c r="D7" s="27" t="s">
+        <v>49</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="H7" s="33" t="s">
-        <v>69</v>
+        <v>97</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1505,20 +1509,20 @@
         <f t="shared" si="2"/>
         <v>46287</v>
       </c>
-      <c r="D8" s="68" t="s">
+      <c r="D8" s="46" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="H8" s="33" t="s">
-        <v>106</v>
+        <v>92</v>
+      </c>
+      <c r="H8" s="32" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1531,7 +1535,7 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="68"/>
+      <c r="D9" s="46"/>
       <c r="E9" s="5" t="s">
         <v>11</v>
       </c>
@@ -1539,10 +1543,10 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="H9" s="33" t="s">
-        <v>70</v>
+        <v>93</v>
+      </c>
+      <c r="H9" s="32" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1554,35 +1558,35 @@
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="69">
+      <c r="C10" s="53">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="65" t="s">
-        <v>60</v>
+      <c r="D10" s="50" t="s">
+        <v>56</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="H10" s="35" t="s">
-        <v>82</v>
+        <v>94</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="49"/>
       <c r="B11" s="48"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="51"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="58" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="60"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
@@ -1594,18 +1598,18 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="66"/>
+      <c r="D12" s="72"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="H12" s="33" t="s">
-        <v>71</v>
+        <v>95</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
@@ -1621,17 +1625,17 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="67"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="H13" s="33"/>
+        <v>96</v>
+      </c>
+      <c r="H13" s="32"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="48"/>
@@ -1643,7 +1647,7 @@
         <f t="shared" si="2"/>
         <v>46304</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="28" t="s">
         <v>39</v>
       </c>
       <c r="E14" s="5" t="s">
@@ -1652,10 +1656,10 @@
       <c r="F14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="H14" s="33"/>
+      <c r="G14" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" s="32"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="47">
@@ -1670,17 +1674,17 @@
         <f t="shared" si="2"/>
         <v>46308</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="29" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="H15" s="34"/>
+      <c r="G15" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H15" s="33"/>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="48"/>
@@ -1692,18 +1696,20 @@
         <f t="shared" si="2"/>
         <v>46311</v>
       </c>
-      <c r="D16" s="28" t="s">
-        <v>49</v>
+      <c r="D16" s="27" t="s">
+        <v>116</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="10"/>
+      <c r="F16" s="10" t="s">
+        <v>118</v>
+      </c>
       <c r="G16" s="21" t="s">
-        <v>103</v>
-      </c>
-      <c r="H16" s="33" t="s">
-        <v>72</v>
+        <v>99</v>
+      </c>
+      <c r="H16" s="32" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1716,13 +1722,13 @@
         <f t="shared" si="2"/>
         <v>46315</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="71"/>
-      <c r="F17" s="72"/>
-      <c r="G17" s="72"/>
-      <c r="H17" s="73"/>
+      <c r="E17" s="55"/>
+      <c r="F17" s="56"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="57"/>
     </row>
     <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="47">
@@ -1736,7 +1742,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="68" t="s">
+      <c r="D18" s="46" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1744,66 +1750,66 @@
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="H18" s="33" t="s">
-        <v>107</v>
+        <v>104</v>
+      </c>
+      <c r="H18" s="32" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
-      <c r="B19" s="61" t="str">
+      <c r="A19" s="49"/>
+      <c r="B19" s="68" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="63">
+      <c r="C19" s="70">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="68"/>
+      <c r="D19" s="46"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="H19" s="33" t="s">
-        <v>73</v>
+        <v>105</v>
+      </c>
+      <c r="H19" s="32" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="48"/>
-      <c r="B20" s="62"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="58" t="s">
-        <v>84</v>
-      </c>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="60"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="65" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="66"/>
+      <c r="G20" s="66"/>
+      <c r="H20" s="67"/>
     </row>
     <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="47">
         <v>9</v>
       </c>
-      <c r="B21" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="C21" s="40">
+      <c r="B21" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="68"/>
-      <c r="E21" s="53" t="s">
-        <v>86</v>
-      </c>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="52" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="52"/>
+      <c r="A22" s="49"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1812,16 +1818,16 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="68"/>
+      <c r="D22" s="46"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="H22" s="33" t="s">
-        <v>74</v>
+        <v>106</v>
+      </c>
+      <c r="H22" s="32" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1834,18 +1840,20 @@
         <f>C19+7</f>
         <v>46329</v>
       </c>
-      <c r="D23" s="28" t="s">
-        <v>50</v>
+      <c r="D23" s="27" t="s">
+        <v>117</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="25"/>
+      <c r="F23" s="73" t="s">
+        <v>119</v>
+      </c>
       <c r="G23" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="H23" s="33" t="s">
-        <v>75</v>
+        <v>107</v>
+      </c>
+      <c r="H23" s="32" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1860,19 +1868,19 @@
         <f t="shared" si="2"/>
         <v>46332</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="25" t="s">
         <v>41</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="H24" s="33"/>
+        <v>108</v>
+      </c>
+      <c r="H24" s="32"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="48"/>
@@ -1884,41 +1892,41 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="68" t="s">
-        <v>64</v>
+      <c r="D25" s="46" t="s">
+        <v>60</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="H25" s="34"/>
+        <v>109</v>
+      </c>
+      <c r="H25" s="33"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="54">
+      <c r="A26" s="61">
         <f>A24+1</f>
         <v>11</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="57" t="s">
-        <v>88</v>
-      </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="55"/>
+      <c r="A27" s="62"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -1927,20 +1935,20 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="68"/>
+      <c r="D27" s="46"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="H27" s="33" t="s">
-        <v>76</v>
+        <v>110</v>
+      </c>
+      <c r="H27" s="32" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="56"/>
+      <c r="A28" s="63"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -1949,18 +1957,20 @@
         <f>C25+7</f>
         <v>46343</v>
       </c>
-      <c r="D28" s="28" t="s">
-        <v>56</v>
+      <c r="D28" s="27" t="s">
+        <v>120</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="21"/>
+      <c r="F28" s="21" t="s">
+        <v>121</v>
+      </c>
       <c r="G28" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="H28" s="33" t="s">
-        <v>80</v>
+        <v>111</v>
+      </c>
+      <c r="H28" s="32" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1976,19 +1986,19 @@
         <f t="shared" si="2"/>
         <v>46346</v>
       </c>
-      <c r="D29" s="26" t="s">
-        <v>119</v>
+      <c r="D29" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="G29" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="H29" s="34"/>
+        <v>61</v>
+      </c>
+      <c r="G29" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H29" s="33"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="48"/>
@@ -2000,20 +2010,20 @@
         <f t="shared" si="2"/>
         <v>46350</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="28" t="s">
         <v>39</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="G30" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="H30" s="33" t="s">
-        <v>77</v>
+        <v>114</v>
+      </c>
+      <c r="G30" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H30" s="32" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -2026,13 +2036,13 @@
         <f t="shared" si="2"/>
         <v>46353</v>
       </c>
-      <c r="D31" s="31" t="s">
+      <c r="D31" s="30" t="s">
         <v>37</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="10"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="33"/>
+      <c r="H31" s="32"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="47">
@@ -2047,17 +2057,17 @@
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
-      <c r="D32" s="30" t="s">
+      <c r="D32" s="29" t="s">
         <v>34</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F32" s="10"/>
-      <c r="G32" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="H32" s="36"/>
+      <c r="G32" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H32" s="35"/>
     </row>
     <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="48"/>
@@ -2069,20 +2079,20 @@
         <f t="shared" si="2"/>
         <v>46360</v>
       </c>
-      <c r="D33" s="26" t="s">
-        <v>58</v>
+      <c r="D33" s="25" t="s">
+        <v>54</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="G33" s="45" t="s">
-        <v>102</v>
-      </c>
-      <c r="H33" s="33" t="s">
-        <v>78</v>
+        <v>62</v>
+      </c>
+      <c r="G33" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="H33" s="32" t="s">
+        <v>74</v>
       </c>
       <c r="I33"/>
     </row>
@@ -2099,18 +2109,20 @@
         <f t="shared" si="2"/>
         <v>46364</v>
       </c>
-      <c r="D34" s="28" t="s">
-        <v>57</v>
+      <c r="D34" s="27" t="s">
+        <v>122</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F34" s="19"/>
-      <c r="G34" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="H34" s="33" t="s">
-        <v>79</v>
+      <c r="F34" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="H34" s="32" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -2123,19 +2135,19 @@
         <f t="shared" si="2"/>
         <v>46367</v>
       </c>
-      <c r="D35" s="26" t="s">
-        <v>58</v>
+      <c r="D35" s="25" t="s">
+        <v>54</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F35" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="G35" s="46" t="s">
-        <v>102</v>
-      </c>
-      <c r="H35" s="34"/>
+      <c r="F35" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="G35" s="45" t="s">
+        <v>98</v>
+      </c>
+      <c r="H35" s="33"/>
     </row>
     <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
@@ -2145,23 +2157,23 @@
       <c r="C36" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D36" s="30" t="s">
-        <v>59</v>
+      <c r="D36" s="29" t="s">
+        <v>55</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="10" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G36" s="21"/>
-      <c r="H36" s="33"/>
+      <c r="H36" s="32"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F37" s="6"/>
-      <c r="H37" s="37"/>
+      <c r="H37" s="36"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D38" s="7" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -2169,20 +2181,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E17:H17"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2199,8 +2197,22 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E17:H17"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
update discussion grading criteria and revise overview schedule date
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F141D352-EC8D-42F3-938C-123F2E056030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF84CB17-AC04-43BE-B7EA-7B45AAEFCB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -223,9 +223,6 @@
     <t>1. Classical search</t>
   </si>
   <si>
-    <t>ThinkingAI1-4 + Turing1950</t>
-  </si>
-  <si>
     <t>homework due + quizzes</t>
   </si>
   <si>
@@ -505,37 +502,40 @@
     <t>Computationalism</t>
   </si>
   <si>
-    <t>updated 9/12/2026</t>
-  </si>
-  <si>
     <t>HW6</t>
   </si>
   <si>
     <t>7. Final project</t>
   </si>
   <si>
-    <t>D1: ThinkingAI5-7</t>
-  </si>
-  <si>
-    <t>D2: ThinkingAI8-10</t>
-  </si>
-  <si>
     <t>D1</t>
   </si>
   <si>
     <t>D2</t>
   </si>
   <si>
-    <t>D3: ThinkingAI11 + searle1980</t>
-  </si>
-  <si>
     <t>D3</t>
   </si>
   <si>
-    <t>D4: ThinkingAI12-14</t>
-  </si>
-  <si>
     <t>D4</t>
+  </si>
+  <si>
+    <t>D1: ThinkingAI1-4 + Turing1950</t>
+  </si>
+  <si>
+    <t>D2: ThinkingAI5-7</t>
+  </si>
+  <si>
+    <t>D3: ThinkingAI8-10</t>
+  </si>
+  <si>
+    <t>D4: ThinkingAI11 + searle1980</t>
+  </si>
+  <si>
+    <t>D5: ThinkingAI12-14</t>
+  </si>
+  <si>
+    <t>updated 9/15/2026</t>
   </si>
 </sst>
 </file>
@@ -786,7 +786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -921,27 +921,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -955,54 +1000,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1313,20 +1310,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7109375" style="37" customWidth="1"/>
-    <col min="9" max="9" width="37.85546875" customWidth="1"/>
+    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.453125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="34.7265625" style="37" customWidth="1"/>
+    <col min="9" max="9" width="37.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -1343,18 +1340,18 @@
         <v>0</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G1" s="41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H1" s="42" t="s">
         <v>42</v>
       </c>
       <c r="I1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="47">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="46">
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
@@ -1363,7 +1360,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="D2" s="64" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1371,12 +1368,12 @@
       </c>
       <c r="F2" s="10"/>
       <c r="G2" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="48"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="47"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
       </c>
@@ -1384,20 +1381,20 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="51"/>
+      <c r="D3" s="66"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H3" s="32" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="47">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="46">
         <f>A2+1</f>
         <v>2</v>
       </c>
@@ -1410,17 +1407,17 @@
         <v>46273</v>
       </c>
       <c r="D4" s="52" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E4" s="52"/>
       <c r="F4" s="52"/>
       <c r="G4" s="21"/>
       <c r="H4" s="32" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="48"/>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="47"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
         <v>Fri</v>
@@ -1429,24 +1426,24 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="67" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H5" s="32" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="47">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="46">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
       </c>
@@ -1458,7 +1455,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="46"/>
+      <c r="D6" s="67"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1466,14 +1463,14 @@
         <v>43</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="48"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="47"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1483,21 +1480,21 @@
         <v>46283</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>49</v>
+        <v>118</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="47">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="46">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
       </c>
@@ -1509,24 +1506,24 @@
         <f t="shared" si="2"/>
         <v>46287</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="67" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H8" s="32" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="48"/>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="47"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1535,7 +1532,7 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="46"/>
+      <c r="D9" s="67"/>
       <c r="E9" s="5" t="s">
         <v>11</v>
       </c>
@@ -1543,53 +1540,53 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H9" s="32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="47">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="46">
         <f>A8+1</f>
         <v>5</v>
       </c>
-      <c r="B10" s="47" t="str">
+      <c r="B10" s="46" t="str">
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="68">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="50" t="s">
-        <v>56</v>
+      <c r="D10" s="64" t="s">
+        <v>55</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H10" s="34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="51"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="48" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="49"/>
-      <c r="B11" s="48"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="58" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="60"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="48"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="47"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
         <v>Fri</v>
@@ -1598,22 +1595,22 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="72"/>
+      <c r="D12" s="65"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H12" s="32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
-      <c r="A13" s="47">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="46">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
       </c>
@@ -1625,20 +1622,20 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="51"/>
+      <c r="D13" s="66"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="48"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="47"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1657,12 +1654,12 @@
         <v>45</v>
       </c>
       <c r="G14" s="43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="47">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="46">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
       </c>
@@ -1682,12 +1679,12 @@
       </c>
       <c r="F15" s="10"/>
       <c r="G15" s="43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H15" s="33"/>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="48"/>
+    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="47"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1697,22 +1694,22 @@
         <v>46311</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1725,13 +1722,13 @@
       <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="55"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="57"/>
-    </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="47">
+      <c r="E17" s="70"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="72"/>
+    </row>
+    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="46">
         <v>8</v>
       </c>
       <c r="B18" s="16" t="str">
@@ -1742,7 +1739,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="67" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1750,66 +1747,66 @@
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="49"/>
-      <c r="B19" s="68" t="str">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="51"/>
+      <c r="B19" s="60" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="70">
+      <c r="C19" s="62">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="46"/>
+      <c r="D19" s="67"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="48"/>
-      <c r="B20" s="69"/>
-      <c r="C20" s="71"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="65" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="47"/>
+      <c r="B20" s="61"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="67"/>
+      <c r="E20" s="57" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="59"/>
+    </row>
+    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="46">
+        <v>9</v>
+      </c>
+      <c r="B21" s="38" t="s">
         <v>80</v>
-      </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="66"/>
-      <c r="H20" s="67"/>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="47">
-        <v>9</v>
-      </c>
-      <c r="B21" s="38" t="s">
-        <v>81</v>
       </c>
       <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="46"/>
+      <c r="D21" s="67"/>
       <c r="E21" s="52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F21" s="52"/>
       <c r="G21" s="52"/>
       <c r="H21" s="52"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="49"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="51"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1818,20 +1815,20 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="46"/>
+      <c r="D22" s="67"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H22" s="32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="48"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="47"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
         <v>Tue</v>
@@ -1841,23 +1838,23 @@
         <v>46329</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="73" t="s">
-        <v>119</v>
+      <c r="F23" s="21" t="s">
+        <v>115</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="47">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="46">
         <v>10</v>
       </c>
       <c r="B24" s="16" t="str">
@@ -1875,15 +1872,15 @@
         <v>22</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="48"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="47"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -1892,41 +1889,41 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="46" t="s">
-        <v>60</v>
+      <c r="D25" s="67" t="s">
+        <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H25" s="33"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="61">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="53">
         <f>A24+1</f>
         <v>11</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="46"/>
-      <c r="E26" s="64" t="s">
-        <v>84</v>
-      </c>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" s="56"/>
+      <c r="G26" s="56"/>
+      <c r="H26" s="56"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="54"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -1935,20 +1932,20 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="46"/>
+      <c r="D27" s="67"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="21" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H27" s="32" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="63"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="55"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -1958,23 +1955,23 @@
         <v>46343</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="47">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="46">
         <f>A26+1</f>
         <v>12</v>
       </c>
@@ -1987,21 +1984,21 @@
         <v>46346</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G29" s="43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H29" s="33"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="48"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="47"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2017,16 +2014,16 @@
         <v>27</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G30" s="43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H30" s="32" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="10"/>
       <c r="B31" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2044,8 +2041,8 @@
       <c r="G31" s="21"/>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="47">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="46">
         <f>A29+1</f>
         <v>13</v>
       </c>
@@ -2065,12 +2062,12 @@
       </c>
       <c r="F32" s="10"/>
       <c r="G32" s="43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H32" s="35"/>
     </row>
-    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="48"/>
+    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="47"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2080,24 +2077,24 @@
         <v>46360</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G33" s="44" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H33" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I33"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="47">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="46">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
       </c>
@@ -2116,17 +2113,17 @@
         <v>30</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G34" s="40" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H34" s="32" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="48"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="47"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2136,20 +2133,20 @@
         <v>46367</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>31</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G35" s="45" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H35" s="33"/>
     </row>
-    <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A36" s="10"/>
       <c r="B36" s="16" t="s">
         <v>35</v>
@@ -2158,29 +2155,43 @@
         <v>38</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F37" s="6"/>
       <c r="H37" s="36"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D38" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D39"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E17:H17"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2197,20 +2208,6 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E17:H17"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update index and readings to include news flash about class location and speaker
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF84CB17-AC04-43BE-B7EA-7B45AAEFCB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC5D9AF-5071-4B21-8F77-5C78F8CE6163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="125">
   <si>
     <t>Class number</t>
   </si>
@@ -278,12 +278,6 @@
   </si>
   <si>
     <t>FP3</t>
-  </si>
-  <si>
-    <t>Turing (1950)</t>
-  </si>
-  <si>
-    <t>Thinking AI, Ch 5</t>
   </si>
   <si>
     <t>Thinking AI, Ch 6</t>
@@ -442,9 +436,6 @@
     <t>Logistic function; Binary cross entropy; SGD for 1D neuron</t>
   </si>
   <si>
-    <t>neural nets in PyTorch</t>
-  </si>
-  <si>
     <t>sustainability (UN SDGs); data center impacts; other sust-AI connections</t>
   </si>
   <si>
@@ -454,9 +445,6 @@
     <t>poster session</t>
   </si>
   <si>
-    <t>Turing test; emergence</t>
-  </si>
-  <si>
     <t>--</t>
   </si>
   <si>
@@ -536,6 +524,123 @@
   </si>
   <si>
     <t>updated 9/15/2026</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>neural nets in PyTorch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Turing test; emergence</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Thinking AI, Ch 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Turing (1950)</t>
+    </r>
+  </si>
+  <si>
+    <t>Data center discussion</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Turing test; emergence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>data center sustainability</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Turing (1950)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.padatacenters.com/
+and 
+https://stoppax1.com/</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -545,7 +650,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,6 +714,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -786,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -921,12 +1048,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -936,12 +1093,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -975,32 +1126,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1310,20 +1440,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.453125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7265625" style="37" customWidth="1"/>
-    <col min="9" max="9" width="37.81640625" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" style="37" customWidth="1"/>
+    <col min="9" max="9" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -1343,15 +1473,15 @@
         <v>49</v>
       </c>
       <c r="G1" s="41" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H1" s="42" t="s">
         <v>42</v>
       </c>
       <c r="I1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="46">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="47">
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
@@ -1360,7 +1490,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="50" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1368,12 +1498,12 @@
       </c>
       <c r="F2" s="10"/>
       <c r="G2" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="47"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="48"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
       </c>
@@ -1381,20 +1511,20 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="66"/>
+      <c r="D3" s="51"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="21" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H3" s="32" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="46">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="47">
         <f>A2+1</f>
         <v>2</v>
       </c>
@@ -1407,17 +1537,17 @@
         <v>46273</v>
       </c>
       <c r="D4" s="52" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E4" s="52"/>
       <c r="F4" s="52"/>
       <c r="G4" s="21"/>
       <c r="H4" s="32" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="47"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="48"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
         <v>Fri</v>
@@ -1426,7 +1556,7 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="46" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1436,14 +1566,14 @@
         <v>50</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H5" s="32" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="46">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="47">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
       </c>
@@ -1455,7 +1585,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="67"/>
+      <c r="D6" s="46"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1463,14 +1593,14 @@
         <v>43</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="47"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="48"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1479,22 +1609,22 @@
         <f t="shared" si="2"/>
         <v>46283</v>
       </c>
-      <c r="D7" s="27" t="s">
-        <v>118</v>
+      <c r="D7" s="73" t="s">
+        <v>122</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="H7" s="32" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="46">
+        <v>123</v>
+      </c>
+      <c r="H7" s="40" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="47">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
       </c>
@@ -1506,7 +1636,7 @@
         <f t="shared" si="2"/>
         <v>46287</v>
       </c>
-      <c r="D8" s="67" t="s">
+      <c r="D8" s="25" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
@@ -1516,14 +1646,14 @@
         <v>51</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H8" s="32" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="47"/>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="48"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1532,7 +1662,9 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="67"/>
+      <c r="D9" s="73" t="s">
+        <v>114</v>
+      </c>
       <c r="E9" s="5" t="s">
         <v>11</v>
       </c>
@@ -1540,26 +1672,26 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="H9" s="32" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="46">
+        <v>120</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="47">
         <f>A8+1</f>
         <v>5</v>
       </c>
-      <c r="B10" s="46" t="str">
+      <c r="B10" s="47" t="str">
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="68">
+      <c r="C10" s="53">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="64" t="s">
+      <c r="D10" s="50" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -1567,26 +1699,26 @@
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="21" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="51"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="69"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="48" t="s">
-        <v>78</v>
-      </c>
-      <c r="F11" s="49"/>
-      <c r="G11" s="49"/>
-      <c r="H11" s="50"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="47"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="49"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="58" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="60"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="48"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
         <v>Fri</v>
@@ -1595,7 +1727,7 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="65"/>
+      <c r="D12" s="72"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
@@ -1603,14 +1735,14 @@
         <v>52</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H12" s="32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="46">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="47">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
       </c>
@@ -1622,7 +1754,7 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="66"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1630,12 +1762,12 @@
         <v>56</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="47"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="48"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1654,12 +1786,12 @@
         <v>45</v>
       </c>
       <c r="G14" s="43" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="46">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="47">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
       </c>
@@ -1679,12 +1811,12 @@
       </c>
       <c r="F15" s="10"/>
       <c r="G15" s="43" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H15" s="33"/>
     </row>
-    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="47"/>
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="48"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1694,22 +1826,22 @@
         <v>46311</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1722,13 +1854,13 @@
       <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="70"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="72"/>
-    </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" s="46">
+      <c r="E17" s="55"/>
+      <c r="F17" s="56"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="57"/>
+    </row>
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="47">
         <v>8</v>
       </c>
       <c r="B18" s="16" t="str">
@@ -1739,7 +1871,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="67" t="s">
+      <c r="D18" s="46" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1747,66 +1879,66 @@
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="21" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="51"/>
-      <c r="B19" s="60" t="str">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="49"/>
+      <c r="B19" s="68" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="62">
+      <c r="C19" s="70">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="67"/>
+      <c r="D19" s="46"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="21" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="47"/>
-      <c r="B20" s="61"/>
-      <c r="C20" s="63"/>
-      <c r="D20" s="67"/>
-      <c r="E20" s="57" t="s">
-        <v>79</v>
-      </c>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="59"/>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="46">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="48"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="66"/>
+      <c r="G20" s="66"/>
+      <c r="H20" s="67"/>
+    </row>
+    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="47">
         <v>9</v>
       </c>
       <c r="B21" s="38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="67"/>
+      <c r="D21" s="46"/>
       <c r="E21" s="52" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F21" s="52"/>
       <c r="G21" s="52"/>
       <c r="H21" s="52"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="51"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="49"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1815,20 +1947,20 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="67"/>
+      <c r="D22" s="46"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="21" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H22" s="32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="47"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="48"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
         <v>Tue</v>
@@ -1838,23 +1970,23 @@
         <v>46329</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="46">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="47">
         <v>10</v>
       </c>
       <c r="B24" s="16" t="str">
@@ -1875,12 +2007,12 @@
         <v>57</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="47"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="48"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -1889,7 +2021,7 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="67" t="s">
+      <c r="D25" s="46" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -1899,31 +2031,31 @@
         <v>58</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="H25" s="33"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="53">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="61">
         <f>A24+1</f>
         <v>11</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="67"/>
-      <c r="E26" s="56" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" s="56"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="56"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="54"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="62"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -1932,20 +2064,20 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="67"/>
+      <c r="D27" s="46"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="21" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H27" s="32" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="55"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="63"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -1955,23 +2087,23 @@
         <v>46343</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="46">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="47">
         <f>A26+1</f>
         <v>12</v>
       </c>
@@ -1984,7 +2116,7 @@
         <v>46346</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>26</v>
@@ -1993,12 +2125,12 @@
         <v>60</v>
       </c>
       <c r="G29" s="43" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H29" s="33"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="47"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="48"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2014,16 +2146,16 @@
         <v>27</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G30" s="43" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H30" s="32" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2041,8 +2173,8 @@
       <c r="G31" s="21"/>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="46">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="47">
         <f>A29+1</f>
         <v>13</v>
       </c>
@@ -2062,12 +2194,12 @@
       </c>
       <c r="F32" s="10"/>
       <c r="G32" s="43" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H32" s="35"/>
     </row>
-    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="47"/>
+    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="48"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2086,15 +2218,15 @@
         <v>61</v>
       </c>
       <c r="G33" s="44" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H33" s="32" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I33"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="46">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="47">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
       </c>
@@ -2107,23 +2239,23 @@
         <v>46364</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G34" s="40" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H34" s="32" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="47"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="48"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2142,11 +2274,11 @@
         <v>62</v>
       </c>
       <c r="G35" s="45" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H35" s="33"/>
     </row>
-    <row r="36" spans="1:9" ht="39" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="16" t="s">
         <v>35</v>
@@ -2164,34 +2296,20 @@
       <c r="G36" s="21"/>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F37" s="6"/>
       <c r="H37" s="36"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D38" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D39"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E17:H17"/>
+  <mergeCells count="29">
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2208,6 +2326,19 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E17:H17"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update overview schedule link and add new class details to resources
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC5D9AF-5071-4B21-8F77-5C78F8CE6163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE2EB0C-1323-4E46-9259-9C6EECEE08DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -523,9 +523,6 @@
     <t>D5: ThinkingAI12-14</t>
   </si>
   <si>
-    <t>updated 9/15/2026</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <strike/>
@@ -641,6 +638,9 @@
 and 
 https://stoppax1.com/</t>
     </r>
+  </si>
+  <si>
+    <t>updated 9/22/2026</t>
   </si>
 </sst>
 </file>
@@ -1048,27 +1048,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1083,54 +1131,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1440,20 +1440,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7109375" style="37" customWidth="1"/>
-    <col min="9" max="9" width="37.85546875" customWidth="1"/>
+    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.453125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="34.7265625" style="37" customWidth="1"/>
+    <col min="9" max="9" width="37.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="I1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="47">
         <v>1</v>
       </c>
@@ -1490,7 +1490,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="D2" s="65" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="48"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
@@ -1511,7 +1511,7 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="51"/>
+      <c r="D3" s="67"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="47">
         <f>A2+1</f>
         <v>2</v>
@@ -1536,17 +1536,17 @@
         <f>C2+7</f>
         <v>46273</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
       <c r="G4" s="21"/>
       <c r="H4" s="32" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="48"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
@@ -1556,7 +1556,7 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="68" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1572,7 +1572,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="47">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
@@ -1585,7 +1585,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="46"/>
+      <c r="D6" s="68"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="48"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1609,21 +1609,21 @@
         <f t="shared" si="2"/>
         <v>46283</v>
       </c>
-      <c r="D7" s="73" t="s">
-        <v>122</v>
+      <c r="D7" s="46" t="s">
+        <v>121</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="H7" s="40" t="s">
         <v>123</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="47">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
@@ -1652,7 +1652,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="48"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1662,7 +1662,7 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="73" t="s">
+      <c r="D9" s="46" t="s">
         <v>114</v>
       </c>
       <c r="E9" s="5" t="s">
@@ -1672,13 +1672,13 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="H9" s="33" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="47">
         <f>A8+1</f>
         <v>5</v>
@@ -1687,11 +1687,11 @@
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="69">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="50" t="s">
+      <c r="D10" s="65" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -1705,19 +1705,19 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="49"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="52"/>
       <c r="B11" s="48"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="58" t="s">
+      <c r="C11" s="70"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="60"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F11" s="50"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="51"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
@@ -1727,7 +1727,7 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="72"/>
+      <c r="D12" s="66"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
       <c r="A13" s="47">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
@@ -1754,7 +1754,7 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="51"/>
+      <c r="D13" s="67"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="48"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="47">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H15" s="33"/>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="48"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1841,7 +1841,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1854,12 +1854,12 @@
       <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="55"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="57"/>
-    </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="E17" s="71"/>
+      <c r="F17" s="72"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="73"/>
+    </row>
+    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="47">
         <v>8</v>
       </c>
@@ -1871,7 +1871,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="68" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1885,17 +1885,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="49"/>
-      <c r="B19" s="68" t="str">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="52"/>
+      <c r="B19" s="61" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="70">
+      <c r="C19" s="63">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="46"/>
+      <c r="D19" s="68"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
@@ -1907,19 +1907,19 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="48"/>
-      <c r="B20" s="69"/>
-      <c r="C20" s="71"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="65" t="s">
+      <c r="B20" s="62"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="58" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="66"/>
-      <c r="H20" s="67"/>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="60"/>
+    </row>
+    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="47">
         <v>9</v>
       </c>
@@ -1929,16 +1929,16 @@
       <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="52" t="s">
+      <c r="D21" s="68"/>
+      <c r="E21" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="52"/>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="49"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="52"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1947,7 +1947,7 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="46"/>
+      <c r="D22" s="68"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="48"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
@@ -1985,7 +1985,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="47">
         <v>10</v>
       </c>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="48"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2021,7 +2021,7 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="68" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -2035,8 +2035,8 @@
       </c>
       <c r="H25" s="33"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="61">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="54">
         <f>A24+1</f>
         <v>11</v>
       </c>
@@ -2046,16 +2046,16 @@
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="46"/>
-      <c r="E26" s="64" t="s">
+      <c r="D26" s="68"/>
+      <c r="E26" s="57" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="55"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -2064,7 +2064,7 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="46"/>
+      <c r="D27" s="68"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
@@ -2076,8 +2076,8 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="63"/>
+    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="56"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -2102,7 +2102,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="47">
         <f>A26+1</f>
         <v>12</v>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H29" s="33"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="48"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2155,7 +2155,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="10"/>
       <c r="B31" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2173,7 +2173,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="47">
         <f>A29+1</f>
         <v>13</v>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="H32" s="35"/>
     </row>
-    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="48"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="I33"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="47">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
@@ -2254,7 +2254,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="48"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="H35" s="33"/>
     </row>
-    <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A36" s="10"/>
       <c r="B36" s="16" t="s">
         <v>35</v>
@@ -2296,20 +2296,33 @@
       <c r="G36" s="21"/>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F37" s="6"/>
       <c r="H37" s="36"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D38" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D39"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E17:H17"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2326,19 +2339,6 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E17:H17"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: update course overview schedule to version 10-16-2026
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE2EB0C-1323-4E46-9259-9C6EECEE08DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B792BF8E-6E63-46FC-BDAD-69B5DDB5A676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -496,9 +496,6 @@
     <t>7. Final project</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>D2</t>
   </si>
   <si>
@@ -640,7 +637,10 @@
     </r>
   </si>
   <si>
-    <t>updated 9/22/2026</t>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>updated 10/16/2026</t>
   </si>
 </sst>
 </file>
@@ -913,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1051,12 +1051,42 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1066,12 +1096,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1105,32 +1129,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1481,7 +1484,7 @@
       <c r="I1"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="47">
+      <c r="A2" s="48">
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
@@ -1490,7 +1493,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="65" t="s">
+      <c r="D2" s="51" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1503,7 +1506,7 @@
       <c r="H2" s="32"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="48"/>
+      <c r="A3" s="49"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
       </c>
@@ -1511,7 +1514,7 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="67"/>
+      <c r="D3" s="52"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
@@ -1524,7 +1527,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="47">
+      <c r="A4" s="48">
         <f>A2+1</f>
         <v>2</v>
       </c>
@@ -1547,7 +1550,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="48"/>
+      <c r="A5" s="49"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
         <v>Fri</v>
@@ -1556,7 +1559,7 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="68" t="s">
+      <c r="D5" s="47" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1573,7 +1576,7 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="47">
+      <c r="A6" s="48">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
       </c>
@@ -1585,7 +1588,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="68"/>
+      <c r="D6" s="47"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1600,7 +1603,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="48"/>
+      <c r="A7" s="49"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1610,21 +1613,21 @@
         <v>46283</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="H7" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>123</v>
-      </c>
     </row>
     <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="47">
+      <c r="A8" s="48">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
       </c>
@@ -1653,7 +1656,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="48"/>
+      <c r="A9" s="49"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1663,7 +1666,7 @@
         <v>46290</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>11</v>
@@ -1672,26 +1675,26 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="H9" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="H9" s="33" t="s">
-        <v>120</v>
-      </c>
     </row>
     <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="47">
+      <c r="A10" s="48">
         <f>A8+1</f>
         <v>5</v>
       </c>
-      <c r="B10" s="47" t="str">
+      <c r="B10" s="48" t="str">
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="69">
+      <c r="C10" s="54">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="65" t="s">
+      <c r="D10" s="51" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -1706,19 +1709,19 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="52"/>
-      <c r="B11" s="48"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="49" t="s">
+      <c r="A11" s="50"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="51"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="61"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="48"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
         <v>Fri</v>
@@ -1727,7 +1730,7 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="66"/>
+      <c r="D12" s="73"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
@@ -1742,7 +1745,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="47">
+      <c r="A13" s="48">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
       </c>
@@ -1754,7 +1757,7 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="67"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1767,7 +1770,7 @@
       <c r="H13" s="32"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="48"/>
+      <c r="A14" s="49"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1791,7 +1794,7 @@
       <c r="H14" s="32"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="47">
+      <c r="A15" s="48">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
       </c>
@@ -1816,7 +1819,7 @@
       <c r="H15" s="33"/>
     </row>
     <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="48"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1826,7 +1829,7 @@
         <v>46311</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
@@ -1854,13 +1857,13 @@
       <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="71"/>
-      <c r="F17" s="72"/>
-      <c r="G17" s="72"/>
-      <c r="H17" s="73"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="58"/>
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" s="47">
+      <c r="A18" s="48">
         <v>8</v>
       </c>
       <c r="B18" s="16" t="str">
@@ -1871,7 +1874,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="68" t="s">
+      <c r="D18" s="47" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1886,16 +1889,16 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="52"/>
-      <c r="B19" s="61" t="str">
+      <c r="A19" s="50"/>
+      <c r="B19" s="69" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="63">
+      <c r="C19" s="71">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="68"/>
+      <c r="D19" s="47"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
@@ -1908,19 +1911,19 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="48"/>
-      <c r="B20" s="62"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="58" t="s">
+      <c r="A20" s="49"/>
+      <c r="B20" s="70"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="66" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="60"/>
+      <c r="F20" s="67"/>
+      <c r="G20" s="67"/>
+      <c r="H20" s="68"/>
     </row>
     <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="47">
+      <c r="A21" s="48">
         <v>9</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1929,7 +1932,7 @@
       <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="68"/>
+      <c r="D21" s="47"/>
       <c r="E21" s="53" t="s">
         <v>79</v>
       </c>
@@ -1938,7 +1941,7 @@
       <c r="H21" s="53"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="52"/>
+      <c r="A22" s="50"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1947,7 +1950,7 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="68"/>
+      <c r="D22" s="47"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
@@ -1960,7 +1963,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="48"/>
+      <c r="A23" s="49"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
         <v>Tue</v>
@@ -1970,7 +1973,7 @@
         <v>46329</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
@@ -1986,7 +1989,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="47">
+      <c r="A24" s="48">
         <v>10</v>
       </c>
       <c r="B24" s="16" t="str">
@@ -2012,7 +2015,7 @@
       <c r="H24" s="32"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="48"/>
+      <c r="A25" s="49"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2021,7 +2024,7 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="68" t="s">
+      <c r="D25" s="47" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -2036,7 +2039,7 @@
       <c r="H25" s="33"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="54">
+      <c r="A26" s="62">
         <f>A24+1</f>
         <v>11</v>
       </c>
@@ -2046,16 +2049,16 @@
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="57" t="s">
+      <c r="D26" s="47"/>
+      <c r="E26" s="65" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="55"/>
+      <c r="A27" s="63"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -2064,7 +2067,7 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="68"/>
+      <c r="D27" s="47"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
@@ -2077,7 +2080,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="56"/>
+      <c r="A28" s="64"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -2087,7 +2090,7 @@
         <v>46343</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
@@ -2103,7 +2106,7 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="47">
+      <c r="A29" s="48">
         <f>A26+1</f>
         <v>12</v>
       </c>
@@ -2130,7 +2133,7 @@
       <c r="H29" s="33"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="48"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2174,7 +2177,7 @@
       <c r="H31" s="32"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="47">
+      <c r="A32" s="48">
         <f>A29+1</f>
         <v>13</v>
       </c>
@@ -2199,7 +2202,7 @@
       <c r="H32" s="35"/>
     </row>
     <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="48"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2226,7 +2229,7 @@
       <c r="I33"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="47">
+      <c r="A34" s="48">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
       </c>
@@ -2239,13 +2242,13 @@
         <v>46364</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="G34" s="40" t="s">
         <v>107</v>
@@ -2255,7 +2258,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="48"/>
+      <c r="A35" s="49"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2297,32 +2300,17 @@
       <c r="H36" s="32"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" s="74" t="s">
+        <v>124</v>
+      </c>
       <c r="F37" s="6"/>
       <c r="H37" s="36"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D38" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D39"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E17:H17"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A35"/>
@@ -2339,6 +2327,19 @@
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D10:D13"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E17:H17"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: update overview schedule link to version 10-22-2026
</commit_message>
<xml_diff>
--- a/comp364-schedule.xlsx
+++ b/comp364-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B792BF8E-6E63-46FC-BDAD-69B5DDB5A676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF2916C-1AA7-4C99-BD1F-35EDC413755F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -463,12 +463,6 @@
     <t>Matrix Algebra, Sec 6 and Sec 7</t>
   </si>
   <si>
-    <t>Computing convolutions and their output sizes; regression via MSE</t>
-  </si>
-  <si>
-    <t>CNNs in PyTorch</t>
-  </si>
-  <si>
     <t>optional lab day</t>
   </si>
   <si>
@@ -640,7 +634,13 @@
     <t>D5</t>
   </si>
   <si>
-    <t>updated 10/16/2026</t>
+    <t>Computing convolutions and their output sizes</t>
+  </si>
+  <si>
+    <t>regression via MSE; CNNs in PyTorch</t>
+  </si>
+  <si>
+    <t>updated 10/22/2026</t>
   </si>
 </sst>
 </file>
@@ -1051,6 +1051,9 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1131,9 +1134,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1443,20 +1443,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.453125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34.7265625" style="37" customWidth="1"/>
-    <col min="9" max="9" width="37.81640625" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.42578125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" style="37" customWidth="1"/>
+    <col min="9" max="9" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -1483,8 +1483,8 @@
       </c>
       <c r="I1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="48">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="49">
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
@@ -1493,7 +1493,7 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="D2" s="52" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -1505,8 +1505,8 @@
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="49"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="50"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
       </c>
@@ -1514,7 +1514,7 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="52"/>
+      <c r="D3" s="53"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
@@ -1526,8 +1526,8 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="48">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="49">
         <f>A2+1</f>
         <v>2</v>
       </c>
@@ -1539,18 +1539,18 @@
         <f>C2+7</f>
         <v>46273</v>
       </c>
-      <c r="D4" s="53" t="s">
+      <c r="D4" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
       <c r="G4" s="21"/>
       <c r="H4" s="32" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="49"/>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="50"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
         <v>Fri</v>
@@ -1559,7 +1559,7 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="48" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1575,8 +1575,8 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="48">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="49">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
       </c>
@@ -1588,7 +1588,7 @@
         <f t="shared" ref="C6:C35" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="47"/>
+      <c r="D6" s="48"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
@@ -1602,8 +1602,8 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="49"/>
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="50"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1613,21 +1613,21 @@
         <v>46283</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H7" s="40" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="48">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="49">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
       </c>
@@ -1655,8 +1655,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="49"/>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="50"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1666,7 +1666,7 @@
         <v>46290</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>11</v>
@@ -1675,26 +1675,26 @@
         <v>44</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="48">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="49">
         <f>A8+1</f>
         <v>5</v>
       </c>
-      <c r="B10" s="48" t="str">
+      <c r="B10" s="49" t="str">
         <f>B8</f>
         <v>Tue</v>
       </c>
-      <c r="C10" s="54">
+      <c r="C10" s="55">
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D10" s="51" t="s">
+      <c r="D10" s="52" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -1708,20 +1708,20 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="50"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="59" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="51"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="56"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="61"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="49"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="62"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="50"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
         <v>Fri</v>
@@ -1730,7 +1730,7 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="73"/>
+      <c r="D12" s="74"/>
       <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
@@ -1744,8 +1744,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="48">
+    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="49">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
       </c>
@@ -1757,7 +1757,7 @@
         <f>C10+7</f>
         <v>46301</v>
       </c>
-      <c r="D13" s="52"/>
+      <c r="D13" s="53"/>
       <c r="E13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1769,8 +1769,8 @@
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="49"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="50"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1793,8 +1793,8 @@
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="48">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="49">
         <f t="shared" ref="A15" si="5">A13+1</f>
         <v>7</v>
       </c>
@@ -1818,8 +1818,8 @@
       </c>
       <c r="H15" s="33"/>
     </row>
-    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="49"/>
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="50"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -1829,13 +1829,13 @@
         <v>46311</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G16" s="21" t="s">
         <v>94</v>
@@ -1844,7 +1844,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1857,13 +1857,13 @@
       <c r="D17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="56"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="58"/>
-    </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" s="48">
+      <c r="E17" s="57"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="59"/>
+    </row>
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="49">
         <v>8</v>
       </c>
       <c r="B18" s="16" t="str">
@@ -1874,7 +1874,7 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="47" t="s">
+      <c r="D18" s="48" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="5" t="s">
@@ -1882,48 +1882,48 @@
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="21" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="H18" s="32" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="50"/>
-      <c r="B19" s="69" t="str">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="51"/>
+      <c r="B19" s="70" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="71">
+      <c r="C19" s="72">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="47"/>
+      <c r="D19" s="48"/>
       <c r="E19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="21" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="H19" s="32" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="49"/>
-      <c r="B20" s="70"/>
-      <c r="C20" s="72"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="66" t="s">
+    <row r="20" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="50"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="73"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="68"/>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="48">
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="69"/>
+    </row>
+    <row r="21" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="49">
         <v>9</v>
       </c>
       <c r="B21" s="38" t="s">
@@ -1932,16 +1932,16 @@
       <c r="C21" s="39">
         <v>46324</v>
       </c>
-      <c r="D21" s="47"/>
-      <c r="E21" s="53" t="s">
+      <c r="D21" s="48"/>
+      <c r="E21" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="50"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="51"/>
       <c r="B22" s="16" t="str">
         <f>B18</f>
         <v>Fri</v>
@@ -1950,20 +1950,20 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D22" s="47"/>
+      <c r="D22" s="48"/>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H22" s="32" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="49"/>
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="50"/>
       <c r="B23" s="16" t="str">
         <f>B19</f>
         <v>Tue</v>
@@ -1973,23 +1973,23 @@
         <v>46329</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H23" s="32" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="48">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="49">
         <v>10</v>
       </c>
       <c r="B24" s="16" t="str">
@@ -2010,12 +2010,12 @@
         <v>57</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="49"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="50"/>
       <c r="B25" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2024,7 +2024,7 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D25" s="47" t="s">
+      <c r="D25" s="48" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -2034,12 +2034,12 @@
         <v>58</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H25" s="33"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="62">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="63">
         <f>A24+1</f>
         <v>11</v>
       </c>
@@ -2049,16 +2049,16 @@
       <c r="C26" s="14">
         <v>46337</v>
       </c>
-      <c r="D26" s="47"/>
-      <c r="E26" s="65" t="s">
+      <c r="D26" s="48"/>
+      <c r="E26" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="65"/>
-      <c r="G26" s="65"/>
-      <c r="H26" s="65"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="63"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="64"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>
         <v>Fri</v>
@@ -2067,20 +2067,20 @@
         <f>C24+7</f>
         <v>46339</v>
       </c>
-      <c r="D27" s="47"/>
+      <c r="D27" s="48"/>
       <c r="E27" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H27" s="32" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="64"/>
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="65"/>
       <c r="B28" s="16" t="str">
         <f>B25</f>
         <v>Tue</v>
@@ -2090,23 +2090,23 @@
         <v>46343</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H28" s="32" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="48">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="49">
         <f>A26+1</f>
         <v>12</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>46346</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>26</v>
@@ -2132,8 +2132,8 @@
       </c>
       <c r="H29" s="33"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="49"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="50"/>
       <c r="B30" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Tue</v>
@@ -2149,7 +2149,7 @@
         <v>27</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G30" s="43" t="s">
         <v>93</v>
@@ -2158,7 +2158,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="16" t="str">
         <f t="shared" si="1"/>
@@ -2176,8 +2176,8 @@
       <c r="G31" s="21"/>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="48">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="49">
         <f>A29+1</f>
         <v>13</v>
       </c>
@@ -2201,8 +2201,8 @@
       </c>
       <c r="H32" s="35"/>
     </row>
-    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="49"/>
+    <row r="33" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="50"/>
       <c r="B33" s="17" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2228,8 +2228,8 @@
       </c>
       <c r="I33"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="48">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="49">
         <f t="shared" ref="A34" si="6">A32+1</f>
         <v>14</v>
       </c>
@@ -2242,23 +2242,23 @@
         <v>46364</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G34" s="40" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H34" s="32" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="49"/>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="50"/>
       <c r="B35" s="16" t="str">
         <f t="shared" si="1"/>
         <v>Fri</v>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="H35" s="33"/>
     </row>
-    <row r="36" spans="1:9" ht="39" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="16" t="s">
         <v>35</v>
@@ -2299,14 +2299,14 @@
       <c r="G36" s="21"/>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" s="74" t="s">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="47" t="s">
         <v>124</v>
       </c>
       <c r="F37" s="6"/>
       <c r="H37" s="36"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D39"/>
     </row>
   </sheetData>

</xml_diff>